<commit_message>
docs(relatorio): atualiza planilha consolidada DADOS_CONSOLIDADOS_TCC.xlsx com dados finais AWS e Local
</commit_message>
<xml_diff>
--- a/relatorio/DADOS_CONSOLIDADOS_TCC.xlsx
+++ b/relatorio/DADOS_CONSOLIDADOS_TCC.xlsx
@@ -611,25 +611,25 @@
         <v>3</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>45.1</v>
+        <v>43.81</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>3.63</v>
+        <v>4.41</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>443.8</v>
+        <v>457.8</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>29.7</v>
+        <v>40.5</v>
       </c>
       <c r="H6" s="7" t="n">
-        <v>446.7</v>
+        <v>460.5</v>
       </c>
       <c r="I6" s="7" t="n">
-        <v>570</v>
+        <v>615.1</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>855.5</v>
+        <v>654.5</v>
       </c>
       <c r="K6" s="6" t="inlineStr">
         <is>
@@ -657,34 +657,34 @@
         <v>3</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>129.53</v>
+        <v>503.93</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>11.68</v>
+        <v>634.98</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>146</v>
+        <v>98.90000000000001</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>13.9</v>
+        <v>70.5</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>156.2</v>
+        <v>133.5</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>182.6</v>
+        <v>126.6</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>192.6</v>
+        <v>141.8</v>
       </c>
       <c r="K7" s="6" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>33.33%</t>
         </is>
       </c>
       <c r="L7" s="6" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>66.7%</t>
         </is>
       </c>
     </row>
@@ -703,25 +703,25 @@
         <v>3</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>44.35</v>
+        <v>47.18</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>7.53</v>
+        <v>0.8</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>1083.6</v>
+        <v>1003.8</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>194</v>
+        <v>17.2</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>1008.1</v>
+        <v>1031.2</v>
       </c>
       <c r="I8" s="7" t="n">
-        <v>1747.8</v>
+        <v>1244.8</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>1889</v>
+        <v>1295.4</v>
       </c>
       <c r="K8" s="6" t="inlineStr">
         <is>
@@ -749,34 +749,34 @@
         <v>3</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>105.14</v>
+        <v>554.13</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>30.58</v>
+        <v>874.35</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>456.4</v>
+        <v>1052.3</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>112.8</v>
+        <v>1385.5</v>
       </c>
       <c r="H9" s="7" t="n">
         <v>528.3</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>659.9</v>
+        <v>2268.2</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>684</v>
+        <v>2279.1</v>
       </c>
       <c r="K9" s="6" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>33.33%</t>
         </is>
       </c>
       <c r="L9" s="6" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>66.7%</t>
         </is>
       </c>
     </row>
@@ -795,25 +795,25 @@
         <v>3</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>47.2</v>
+        <v>43.24</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>2.01</v>
+        <v>4.02</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>1999.5</v>
+        <v>2168.4</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>117.5</v>
+        <v>167.6</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>2031.9</v>
+        <v>2127.4</v>
       </c>
       <c r="I10" s="7" t="n">
-        <v>2627.1</v>
+        <v>3229.6</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>2747.3</v>
+        <v>3429.5</v>
       </c>
       <c r="K10" s="6" t="inlineStr">
         <is>
@@ -841,34 +841,34 @@
         <v>3</v>
       </c>
       <c r="D11" s="7" t="n">
-        <v>90.65000000000001</v>
+        <v>485.77</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>5.31</v>
+        <v>750.87</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>1003.3</v>
+        <v>1496.2</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>67.7</v>
+        <v>1770.7</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>1093.2</v>
+        <v>1017.2</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>1386.2</v>
+        <v>2519.1</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>1426.2</v>
+        <v>2546.9</v>
       </c>
       <c r="K11" s="6" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>33.33%</t>
         </is>
       </c>
       <c r="L11" s="6" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>66.7%</t>
         </is>
       </c>
     </row>
@@ -944,16 +944,16 @@
         <v>3</v>
       </c>
       <c r="D16" s="7" t="n">
-        <v>13.7</v>
+        <v>16.38</v>
       </c>
       <c r="E16" s="7" t="n">
-        <v>5.65</v>
+        <v>1.63</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>369.9</v>
+        <v>318.7</v>
       </c>
       <c r="G16" s="7" t="n">
-        <v>833</v>
+        <v>582.4</v>
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
@@ -976,20 +976,20 @@
         <v>3</v>
       </c>
       <c r="D17" s="7" t="n">
-        <v>69.23</v>
+        <v>81.81</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>5.01</v>
+        <v>34.2</v>
       </c>
       <c r="F17" s="7" t="n">
-        <v>75.5</v>
+        <v>55.1</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>133</v>
+        <v>127.9</v>
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>66.7%</t>
         </is>
       </c>
     </row>
@@ -1008,16 +1008,16 @@
         <v>3</v>
       </c>
       <c r="D18" s="7" t="n">
-        <v>5.24</v>
+        <v>14.14</v>
       </c>
       <c r="E18" s="7" t="n">
-        <v>2.18</v>
+        <v>6.46</v>
       </c>
       <c r="F18" s="7" t="n">
-        <v>365</v>
+        <v>374.5</v>
       </c>
       <c r="G18" s="7" t="n">
-        <v>3869.9</v>
+        <v>1242.3</v>
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
@@ -1040,20 +1040,20 @@
         <v>3</v>
       </c>
       <c r="D19" s="7" t="n">
-        <v>97.8</v>
+        <v>101.15</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>13.31</v>
+        <v>32.2</v>
       </c>
       <c r="F19" s="7" t="n">
-        <v>126.7</v>
+        <v>111.2</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>184.1</v>
+        <v>188.2</v>
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>66.7%</t>
         </is>
       </c>
     </row>
@@ -1072,16 +1072,16 @@
         <v>3</v>
       </c>
       <c r="D20" s="7" t="n">
-        <v>9.43</v>
+        <v>10.59</v>
       </c>
       <c r="E20" s="7" t="n">
-        <v>4.19</v>
+        <v>4.81</v>
       </c>
       <c r="F20" s="7" t="n">
-        <v>578.3</v>
+        <v>500.7</v>
       </c>
       <c r="G20" s="7" t="n">
-        <v>3556.1</v>
+        <v>3731.2</v>
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
@@ -1104,20 +1104,20 @@
         <v>3</v>
       </c>
       <c r="D21" s="7" t="n">
-        <v>73.23999999999999</v>
+        <v>105.06</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>6.27</v>
+        <v>41.19</v>
       </c>
       <c r="F21" s="7" t="n">
-        <v>314.9</v>
+        <v>287</v>
       </c>
       <c r="G21" s="7" t="n">
-        <v>389.2</v>
+        <v>346.1</v>
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>66.7%</t>
         </is>
       </c>
     </row>
@@ -1175,20 +1175,20 @@
         </is>
       </c>
       <c r="B26" s="7" t="n">
-        <v>1643.6</v>
+        <v>10774.8</v>
       </c>
       <c r="C26" s="7" t="n">
-        <v>62.8</v>
+        <v>66.7</v>
       </c>
       <c r="D26" s="7" t="n">
-        <v>655.3</v>
+        <v>5824.4</v>
       </c>
       <c r="E26" s="7" t="n">
-        <v>54.2</v>
+        <v>18.1</v>
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>Excelente (&lt; 2.5s)</t>
+          <t>Aceitável</t>
         </is>
       </c>
     </row>
@@ -1199,16 +1199,16 @@
         </is>
       </c>
       <c r="B27" s="7" t="n">
-        <v>2247.2</v>
+        <v>2111</v>
       </c>
       <c r="C27" s="7" t="n">
-        <v>208.7</v>
+        <v>226</v>
       </c>
       <c r="D27" s="7" t="n">
-        <v>831.2</v>
+        <v>608.2</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>128.6</v>
+        <v>64.3</v>
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
@@ -1368,7 +1368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -1514,25 +1514,25 @@
         <v>100</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D6" s="7" t="n">
         <v>600</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>49.21259842519685</v>
+        <v>44.73272198613286</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>1894.060533333333</v>
+        <v>2075.95505</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>2010.185</v>
+        <v>2155.465</v>
       </c>
       <c r="H6" s="7" t="n">
-        <v>2182.9495</v>
+        <v>2672.6005</v>
       </c>
       <c r="I6" s="7" t="n">
-        <v>2221.8128</v>
+        <v>2773.7543</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>0</v>
@@ -1542,7 +1542,7 @@
       </c>
       <c r="L6" s="6" t="inlineStr">
         <is>
-          <t>benchmark_aws_100users_run2_1789182114397.csv</t>
+          <t>benchmark_aws_100users_run1_1790891018211.csv</t>
         </is>
       </c>
     </row>
@@ -1556,25 +1556,25 @@
         <v>100</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D7" s="7" t="n">
         <v>600</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>45.18752824220515</v>
+        <v>49.21259842519685</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>2126.25435</v>
+        <v>1894.060533333333</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>2061.96</v>
+        <v>2010.185</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>3084.699999999999</v>
+        <v>2182.9495</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>3338.0876</v>
+        <v>2221.8128</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>0</v>
@@ -1584,7 +1584,7 @@
       </c>
       <c r="L7" s="6" t="inlineStr">
         <is>
-          <t>benchmark_aws_100users_run3_1789182131695.csv</t>
+          <t>benchmark_aws_100users_run2_1789182114397.csv</t>
         </is>
       </c>
     </row>
@@ -1595,28 +1595,28 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>120</v>
+        <v>600</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>41.33654839820875</v>
+        <v>38.61003861003861</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>473.8994166666666</v>
+        <v>2353.063016666667</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>446.685</v>
+        <v>2210.8</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>648.0970000000001</v>
+        <v>4170.622499999999</v>
       </c>
       <c r="I8" s="7" t="n">
-        <v>1390.871100000002</v>
+        <v>4382.9779</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>0</v>
@@ -1626,7 +1626,7 @@
       </c>
       <c r="L8" s="6" t="inlineStr">
         <is>
-          <t>benchmark_aws_20users_run1_1789182038527.csv</t>
+          <t>benchmark_aws_100users_run2_1790891037408.csv</t>
         </is>
       </c>
     </row>
@@ -1637,28 +1637,28 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>120</v>
+        <v>600</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>45.36862003780718</v>
+        <v>45.18752824220515</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>442.9535833333333</v>
+        <v>2126.25435</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>452.29</v>
+        <v>2061.96</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>544.4085</v>
+        <v>3084.699999999999</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>584.2952</v>
+        <v>3338.0876</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>0</v>
@@ -1668,7 +1668,7 @@
       </c>
       <c r="L9" s="6" t="inlineStr">
         <is>
-          <t>benchmark_aws_20users_run2_1789182044824.csv</t>
+          <t>benchmark_aws_100users_run3_1789182131695.csv</t>
         </is>
       </c>
     </row>
@@ -1679,28 +1679,28 @@
         </is>
       </c>
       <c r="B10" s="7" t="n">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="C10" s="7" t="n">
         <v>3</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>120</v>
+        <v>600</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>48.58299595141701</v>
+        <v>45.91368227731864</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>414.4184166666666</v>
+        <v>2025.97875</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>409.895</v>
+        <v>2127.415</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>517.6105</v>
+        <v>2433.4285</v>
       </c>
       <c r="I10" s="7" t="n">
-        <v>591.2635</v>
+        <v>2567.4774</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>0</v>
@@ -1710,7 +1710,7 @@
       </c>
       <c r="L10" s="6" t="inlineStr">
         <is>
-          <t>benchmark_aws_20users_run3_1789182050901.csv</t>
+          <t>benchmark_aws_100users_run3_1790891054335.csv</t>
         </is>
       </c>
     </row>
@@ -1721,28 +1721,28 @@
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="C11" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D11" s="7" t="n">
-        <v>300</v>
+        <v>120</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>35.82517315500358</v>
+        <v>41.33654839820875</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>1304.864433333333</v>
+        <v>473.8994166666666</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>1072.9</v>
+        <v>446.685</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>2802.998</v>
+        <v>648.0970000000001</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>3136.1387</v>
+        <v>1390.871100000002</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>0</v>
@@ -1752,7 +1752,7 @@
       </c>
       <c r="L11" s="6" t="inlineStr">
         <is>
-          <t>benchmark_aws_50users_run1_1789182062860.csv</t>
+          <t>benchmark_aws_20users_run1_1789182038527.csv</t>
         </is>
       </c>
     </row>
@@ -1763,28 +1763,28 @@
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="C12" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D12" s="7" t="n">
-        <v>300</v>
+        <v>120</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>50.1002004008016</v>
+        <v>34.04255319148936</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>942.8475</v>
+        <v>583.9791666666666</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>982.255</v>
+        <v>489.625</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>1116.208</v>
+        <v>997.003</v>
       </c>
       <c r="I12" s="7" t="n">
-        <v>1145.3729</v>
+        <v>1119.2605</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>0</v>
@@ -1794,7 +1794,7 @@
       </c>
       <c r="L12" s="6" t="inlineStr">
         <is>
-          <t>benchmark_aws_50users_run2_1789182072502.csv</t>
+          <t>benchmark_aws_20users_run1_1790890956378.csv</t>
         </is>
       </c>
     </row>
@@ -1805,28 +1805,28 @@
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="C13" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D13" s="7" t="n">
-        <v>300</v>
+        <v>120</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>47.11795193968902</v>
+        <v>45.36862003780718</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>1002.9697</v>
+        <v>442.9535833333333</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>1008.135</v>
+        <v>452.29</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>1324.0655</v>
+        <v>544.4085</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>1385.4669</v>
+        <v>584.2952</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>0</v>
@@ -1836,39 +1836,39 @@
       </c>
       <c r="L13" s="6" t="inlineStr">
         <is>
-          <t>benchmark_aws_50users_run3_1789182082445.csv</t>
+          <t>benchmark_aws_20users_run2_1789182044824.csv</t>
         </is>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Local (Docker)</t>
+          <t>Nuvem (AWS)</t>
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="C14" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D14" s="7" t="n">
-        <v>600</v>
+        <v>120</v>
       </c>
       <c r="E14" s="7" t="n">
-        <v>86.20689655172414</v>
+        <v>42.96455424274973</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>1061.329666666667</v>
+        <v>464.4041666666666</v>
       </c>
       <c r="G14" s="7" t="n">
-        <v>1157.69</v>
+        <v>460.545</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>1470.321</v>
+        <v>633.828</v>
       </c>
       <c r="I14" s="7" t="n">
-        <v>1523.4707</v>
+        <v>664.7239000000001</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>0</v>
@@ -1878,39 +1878,39 @@
       </c>
       <c r="L14" s="6" t="inlineStr">
         <is>
-          <t>benchmark_local_100users_run1_1789163315322.csv</t>
+          <t>benchmark_aws_20users_run2_1790890962624.csv</t>
         </is>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Local (Docker)</t>
+          <t>Nuvem (AWS)</t>
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="C15" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D15" s="7" t="n">
-        <v>600</v>
+        <v>120</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>89.20606601248885</v>
+        <v>48.58299595141701</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>1019.745516666667</v>
+        <v>414.4184166666666</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>1093.225</v>
+        <v>409.895</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>1339.71</v>
+        <v>517.6105</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>1366.2917</v>
+        <v>591.2635</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>0</v>
@@ -1920,39 +1920,39 @@
       </c>
       <c r="L15" s="6" t="inlineStr">
         <is>
-          <t>benchmark_local_100users_run2_1789163325103.csv</t>
+          <t>benchmark_aws_20users_run3_1789182050901.csv</t>
         </is>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Local (Docker)</t>
+          <t>Nuvem (AWS)</t>
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="C16" s="7" t="n">
         <v>3</v>
       </c>
       <c r="D16" s="7" t="n">
-        <v>600</v>
+        <v>120</v>
       </c>
       <c r="E16" s="7" t="n">
-        <v>96.52509652509652</v>
+        <v>39.88035892323031</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>928.9411</v>
+        <v>494.67475</v>
       </c>
       <c r="G16" s="7" t="n">
-        <v>1017.18</v>
+        <v>471.835</v>
       </c>
       <c r="H16" s="7" t="n">
-        <v>1348.6185</v>
+        <v>693.982</v>
       </c>
       <c r="I16" s="7" t="n">
-        <v>1388.8524</v>
+        <v>707.4675999999999</v>
       </c>
       <c r="J16" s="7" t="n">
         <v>0</v>
@@ -1962,39 +1962,39 @@
       </c>
       <c r="L16" s="6" t="inlineStr">
         <is>
-          <t>benchmark_local_100users_run3_1789163334355.csv</t>
+          <t>benchmark_aws_20users_run3_1790890969094.csv</t>
         </is>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Local (Docker)</t>
+          <t>Nuvem (AWS)</t>
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="C17" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D17" s="7" t="n">
-        <v>120</v>
+        <v>300</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>126.1829652996846</v>
+        <v>35.82517315500358</v>
       </c>
       <c r="F17" s="7" t="n">
-        <v>151.9005</v>
+        <v>1304.864433333333</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>156.22</v>
+        <v>1072.9</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>186.9865</v>
+        <v>2802.998</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>193.8243</v>
+        <v>3136.1387</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>0</v>
@@ -2004,39 +2004,39 @@
       </c>
       <c r="L17" s="6" t="inlineStr">
         <is>
-          <t>benchmark_local_20users_run1_1789163279018.csv</t>
+          <t>benchmark_aws_50users_run1_1789182062860.csv</t>
         </is>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Local (Docker)</t>
+          <t>Nuvem (AWS)</t>
         </is>
       </c>
       <c r="B18" s="7" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="C18" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D18" s="7" t="n">
-        <v>120</v>
+        <v>300</v>
       </c>
       <c r="E18" s="7" t="n">
-        <v>119.8801198801199</v>
+        <v>36.90036900369003</v>
       </c>
       <c r="F18" s="7" t="n">
-        <v>156.0856666666667</v>
+        <v>1330.145666666667</v>
       </c>
       <c r="G18" s="7" t="n">
-        <v>163.645</v>
+        <v>1138.93</v>
       </c>
       <c r="H18" s="7" t="n">
-        <v>194.742</v>
+        <v>2454.8275</v>
       </c>
       <c r="I18" s="7" t="n">
-        <v>208.7417</v>
+        <v>2663.895199999999</v>
       </c>
       <c r="J18" s="7" t="n">
         <v>0</v>
@@ -2046,39 +2046,39 @@
       </c>
       <c r="L18" s="6" t="inlineStr">
         <is>
-          <t>benchmark_local_20users_run2_1789163283075.csv</t>
+          <t>benchmark_aws_50users_run1_1790890981101.csv</t>
         </is>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Local (Docker)</t>
+          <t>Nuvem (AWS)</t>
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="C19" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D19" s="7" t="n">
-        <v>120</v>
+        <v>300</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>142.5178147268409</v>
+        <v>50.1002004008016</v>
       </c>
       <c r="F19" s="7" t="n">
-        <v>130.1470833333333</v>
+        <v>942.8475</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>133.46</v>
+        <v>982.255</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>166.202</v>
+        <v>1116.208</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>175.1681</v>
+        <v>1145.3729</v>
       </c>
       <c r="J19" s="7" t="n">
         <v>0</v>
@@ -2088,39 +2088,39 @@
       </c>
       <c r="L19" s="6" t="inlineStr">
         <is>
-          <t>benchmark_local_20users_run3_1789163286949.csv</t>
+          <t>benchmark_aws_50users_run2_1789182072502.csv</t>
         </is>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Local (Docker)</t>
+          <t>Nuvem (AWS)</t>
         </is>
       </c>
       <c r="B20" s="7" t="n">
         <v>50</v>
       </c>
       <c r="C20" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D20" s="7" t="n">
         <v>300</v>
       </c>
       <c r="E20" s="7" t="n">
-        <v>139.8601398601399</v>
+        <v>48</v>
       </c>
       <c r="F20" s="7" t="n">
-        <v>330.5770666666667</v>
+        <v>987.0077666666665</v>
       </c>
       <c r="G20" s="7" t="n">
-        <v>316.185</v>
+        <v>1031.2</v>
       </c>
       <c r="H20" s="7" t="n">
-        <v>473.993</v>
+        <v>1169.975</v>
       </c>
       <c r="I20" s="7" t="n">
-        <v>493.8226</v>
+        <v>1216.1767</v>
       </c>
       <c r="J20" s="7" t="n">
         <v>0</v>
@@ -2130,39 +2130,39 @@
       </c>
       <c r="L20" s="6" t="inlineStr">
         <is>
-          <t>benchmark_local_50users_run1_1789163292223.csv</t>
+          <t>benchmark_aws_50users_run2_1790890991012.csv</t>
         </is>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Local (Docker)</t>
+          <t>Nuvem (AWS)</t>
         </is>
       </c>
       <c r="B21" s="7" t="n">
         <v>50</v>
       </c>
       <c r="C21" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D21" s="7" t="n">
         <v>300</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>82.23684210526315</v>
+        <v>47.11795193968902</v>
       </c>
       <c r="F21" s="7" t="n">
-        <v>548.6262666666667</v>
+        <v>1002.9697</v>
       </c>
       <c r="G21" s="7" t="n">
-        <v>549.4300000000001</v>
+        <v>1008.135</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>848.922</v>
+        <v>1324.0655</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>880.3430999999999</v>
+        <v>1385.4669</v>
       </c>
       <c r="J21" s="7" t="n">
         <v>0</v>
@@ -2172,14 +2172,14 @@
       </c>
       <c r="L21" s="6" t="inlineStr">
         <is>
-          <t>benchmark_local_50users_run2_1789163299025.csv</t>
+          <t>benchmark_aws_50users_run3_1789182082445.csv</t>
         </is>
       </c>
     </row>
     <row r="22" ht="19" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>Local (Docker)</t>
+          <t>Nuvem (AWS)</t>
         </is>
       </c>
       <c r="B22" s="7" t="n">
@@ -2192,34 +2192,1168 @@
         <v>300</v>
       </c>
       <c r="E22" s="7" t="n">
+        <v>46.41089108910891</v>
+      </c>
+      <c r="F22" s="7" t="n">
+        <v>1021.321333333333</v>
+      </c>
+      <c r="G22" s="7" t="n">
+        <v>1066.65</v>
+      </c>
+      <c r="H22" s="7" t="n">
+        <v>1240.2605</v>
+      </c>
+      <c r="I22" s="7" t="n">
+        <v>1284.5601</v>
+      </c>
+      <c r="J22" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="L22" s="6" t="inlineStr">
+        <is>
+          <t>benchmark_aws_50users_run3_1790891001108.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="19" customHeight="1">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="C23" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="7" t="n">
+        <v>600</v>
+      </c>
+      <c r="E23" s="7" t="n">
+        <v>86.20689655172414</v>
+      </c>
+      <c r="F23" s="7" t="n">
+        <v>1061.329666666667</v>
+      </c>
+      <c r="G23" s="7" t="n">
+        <v>1157.69</v>
+      </c>
+      <c r="H23" s="7" t="n">
+        <v>1470.321</v>
+      </c>
+      <c r="I23" s="7" t="n">
+        <v>1523.4707</v>
+      </c>
+      <c r="J23" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="L23" s="6" t="inlineStr">
+        <is>
+          <t>benchmark_local_100users_run1_1789163315322.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="19" customHeight="1">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="C24" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="7" t="n">
+        <v>600</v>
+      </c>
+      <c r="E24" s="7" t="n">
+        <v>1600</v>
+      </c>
+      <c r="F24" s="7" t="n">
+        <v>61.20261666666666</v>
+      </c>
+      <c r="G24" s="7" t="n">
+        <v>59.52500000000001</v>
+      </c>
+      <c r="H24" s="7" t="n">
+        <v>94.14649999999997</v>
+      </c>
+      <c r="I24" s="7" t="n">
+        <v>105.114</v>
+      </c>
+      <c r="J24" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="K24" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" s="6" t="inlineStr">
+        <is>
+          <t>benchmark_local_100users_run1_1790816157295.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="19" customHeight="1">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="C25" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="7" t="n">
+        <v>600</v>
+      </c>
+      <c r="E25" s="7" t="n">
+        <v>9.117571079064536</v>
+      </c>
+      <c r="F25" s="7" t="n">
+        <v>3637.705116666667</v>
+      </c>
+      <c r="G25" s="7" t="n">
+        <v>3978.175</v>
+      </c>
+      <c r="H25" s="7" t="n">
+        <v>6097.7405</v>
+      </c>
+      <c r="I25" s="7" t="n">
+        <v>6105.780299999999</v>
+      </c>
+      <c r="J25" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="L25" s="6" t="inlineStr">
+        <is>
+          <t>benchmark_local_100users_run1_1790886122765.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="19" customHeight="1">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="C26" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D26" s="7" t="n">
+        <v>600</v>
+      </c>
+      <c r="E26" s="7" t="n">
+        <v>89.20606601248885</v>
+      </c>
+      <c r="F26" s="7" t="n">
+        <v>1019.745516666667</v>
+      </c>
+      <c r="G26" s="7" t="n">
+        <v>1093.225</v>
+      </c>
+      <c r="H26" s="7" t="n">
+        <v>1339.71</v>
+      </c>
+      <c r="I26" s="7" t="n">
+        <v>1366.2917</v>
+      </c>
+      <c r="J26" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="L26" s="6" t="inlineStr">
+        <is>
+          <t>benchmark_local_100users_run2_1789163325103.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="19" customHeight="1">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="C27" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D27" s="7" t="n">
+        <v>600</v>
+      </c>
+      <c r="E27" s="7" t="n">
+        <v>1652.892561983471</v>
+      </c>
+      <c r="F27" s="7" t="n">
+        <v>67.1563</v>
+      </c>
+      <c r="G27" s="7" t="n">
+        <v>68.265</v>
+      </c>
+      <c r="H27" s="7" t="n">
+        <v>110.2855</v>
+      </c>
+      <c r="I27" s="7" t="n">
+        <v>120.4878</v>
+      </c>
+      <c r="J27" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="K27" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" s="6" t="inlineStr">
+        <is>
+          <t>benchmark_local_100users_run2_1790816163075.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="19" customHeight="1">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="C28" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D28" s="7" t="n">
+        <v>600</v>
+      </c>
+      <c r="E28" s="7" t="n">
+        <v>8.83912787271656</v>
+      </c>
+      <c r="F28" s="7" t="n">
+        <v>3423.745833333333</v>
+      </c>
+      <c r="G28" s="7" t="n">
+        <v>4004.255</v>
+      </c>
+      <c r="H28" s="7" t="n">
+        <v>6082.627500000001</v>
+      </c>
+      <c r="I28" s="7" t="n">
+        <v>6090.0829</v>
+      </c>
+      <c r="J28" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="L28" s="6" t="inlineStr">
+        <is>
+          <t>benchmark_local_100users_run2_1790886196427.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="19" customHeight="1">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="C29" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D29" s="7" t="n">
+        <v>600</v>
+      </c>
+      <c r="E29" s="7" t="n">
+        <v>96.52509652509652</v>
+      </c>
+      <c r="F29" s="7" t="n">
+        <v>928.9411</v>
+      </c>
+      <c r="G29" s="7" t="n">
+        <v>1017.18</v>
+      </c>
+      <c r="H29" s="7" t="n">
+        <v>1348.6185</v>
+      </c>
+      <c r="I29" s="7" t="n">
+        <v>1388.8524</v>
+      </c>
+      <c r="J29" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="L29" s="6" t="inlineStr">
+        <is>
+          <t>benchmark_local_100users_run3_1789163334355.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="19" customHeight="1">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="C30" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D30" s="7" t="n">
+        <v>600</v>
+      </c>
+      <c r="E30" s="7" t="n">
+        <v>1351.351351351351</v>
+      </c>
+      <c r="F30" s="7" t="n">
+        <v>78.61483333333332</v>
+      </c>
+      <c r="G30" s="7" t="n">
+        <v>77.46000000000001</v>
+      </c>
+      <c r="H30" s="7" t="n">
+        <v>108.7245</v>
+      </c>
+      <c r="I30" s="7" t="n">
+        <v>148.9359</v>
+      </c>
+      <c r="J30" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="K30" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" s="6" t="inlineStr">
+        <is>
+          <t>benchmark_local_100users_run3_1790816168434.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="19" customHeight="1">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="C31" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D31" s="7" t="n">
+        <v>600</v>
+      </c>
+      <c r="E31" s="7" t="n">
+        <v>9.448521306415545</v>
+      </c>
+      <c r="F31" s="7" t="n">
+        <v>3481.040483333333</v>
+      </c>
+      <c r="G31" s="7" t="n">
+        <v>3907.67</v>
+      </c>
+      <c r="H31" s="7" t="n">
+        <v>6100.032</v>
+      </c>
+      <c r="I31" s="7" t="n">
+        <v>6102.7819</v>
+      </c>
+      <c r="J31" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="L31" s="6" t="inlineStr">
+        <is>
+          <t>benchmark_local_100users_run3_1790886265638.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="19" customHeight="1">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="C32" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="E32" s="7" t="n">
+        <v>126.1829652996846</v>
+      </c>
+      <c r="F32" s="7" t="n">
+        <v>151.9005</v>
+      </c>
+      <c r="G32" s="7" t="n">
+        <v>156.22</v>
+      </c>
+      <c r="H32" s="7" t="n">
+        <v>186.9865</v>
+      </c>
+      <c r="I32" s="7" t="n">
+        <v>193.8243</v>
+      </c>
+      <c r="J32" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="L32" s="6" t="inlineStr">
+        <is>
+          <t>benchmark_local_20users_run1_1789163279018.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="19" customHeight="1">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="C33" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="E33" s="7" t="n">
+        <v>800</v>
+      </c>
+      <c r="F33" s="7" t="n">
+        <v>27.79983333333333</v>
+      </c>
+      <c r="G33" s="7" t="n">
+        <v>23.535</v>
+      </c>
+      <c r="H33" s="7" t="n">
+        <v>54.643</v>
+      </c>
+      <c r="I33" s="7" t="n">
+        <v>57.5022</v>
+      </c>
+      <c r="J33" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="K33" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L33" s="6" t="inlineStr">
+        <is>
+          <t>benchmark_local_20users_run1_1790816124635.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="19" customHeight="1">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="C34" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="E34" s="7" t="n">
+        <v>4.074702886247878</v>
+      </c>
+      <c r="F34" s="7" t="n">
+        <v>1556.711083333333</v>
+      </c>
+      <c r="G34" s="7" t="n">
+        <v>321.975</v>
+      </c>
+      <c r="H34" s="7" t="n">
+        <v>4398.843999999995</v>
+      </c>
+      <c r="I34" s="7" t="n">
+        <v>6138.5515</v>
+      </c>
+      <c r="J34" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="L34" s="6" t="inlineStr">
+        <is>
+          <t>benchmark_local_20users_run1_1790885882176.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="19" customHeight="1">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="C35" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D35" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="E35" s="7" t="n">
+        <v>119.8801198801199</v>
+      </c>
+      <c r="F35" s="7" t="n">
+        <v>156.0856666666667</v>
+      </c>
+      <c r="G35" s="7" t="n">
+        <v>163.645</v>
+      </c>
+      <c r="H35" s="7" t="n">
+        <v>194.742</v>
+      </c>
+      <c r="I35" s="7" t="n">
+        <v>208.7417</v>
+      </c>
+      <c r="J35" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="L35" s="6" t="inlineStr">
+        <is>
+          <t>benchmark_local_20users_run2_1789163283075.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="19" customHeight="1">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="C36" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D36" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="E36" s="7" t="n">
+        <v>1188.118811881188</v>
+      </c>
+      <c r="F36" s="7" t="n">
+        <v>23.29941666666667</v>
+      </c>
+      <c r="G36" s="7" t="n">
+        <v>18.92</v>
+      </c>
+      <c r="H36" s="7" t="n">
+        <v>50.8625</v>
+      </c>
+      <c r="I36" s="7" t="n">
+        <v>52.7821</v>
+      </c>
+      <c r="J36" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="K36" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L36" s="6" t="inlineStr">
+        <is>
+          <t>benchmark_local_20users_run2_1790816130197.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="19" customHeight="1">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="C37" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D37" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="E37" s="7" t="n">
+        <v>16.40016400164001</v>
+      </c>
+      <c r="F37" s="7" t="n">
+        <v>293.5450833333333</v>
+      </c>
+      <c r="G37" s="7" t="n">
+        <v>152.225</v>
+      </c>
+      <c r="H37" s="7" t="n">
+        <v>2427.624</v>
+      </c>
+      <c r="I37" s="7" t="n">
+        <v>2449.736</v>
+      </c>
+      <c r="J37" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K37" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="L37" s="6" t="inlineStr">
+        <is>
+          <t>benchmark_local_20users_run2_1790885895275.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="19" customHeight="1">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="C38" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D38" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="E38" s="7" t="n">
+        <v>142.5178147268409</v>
+      </c>
+      <c r="F38" s="7" t="n">
+        <v>130.1470833333333</v>
+      </c>
+      <c r="G38" s="7" t="n">
+        <v>133.46</v>
+      </c>
+      <c r="H38" s="7" t="n">
+        <v>166.202</v>
+      </c>
+      <c r="I38" s="7" t="n">
+        <v>175.1681</v>
+      </c>
+      <c r="J38" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K38" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="L38" s="6" t="inlineStr">
+        <is>
+          <t>benchmark_local_20users_run3_1789163286949.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="19" customHeight="1">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="C39" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D39" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="E39" s="7" t="n">
+        <v>1237.113402061856</v>
+      </c>
+      <c r="F39" s="7" t="n">
+        <v>18.1505</v>
+      </c>
+      <c r="G39" s="7" t="n">
+        <v>17.535</v>
+      </c>
+      <c r="H39" s="7" t="n">
+        <v>28.237</v>
+      </c>
+      <c r="I39" s="7" t="n">
+        <v>29.9787</v>
+      </c>
+      <c r="J39" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="K39" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L39" s="6" t="inlineStr">
+        <is>
+          <t>benchmark_local_20users_run3_1790816135569.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="19" customHeight="1">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="C40" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D40" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="E40" s="7" t="n">
+        <v>132.15859030837</v>
+      </c>
+      <c r="F40" s="7" t="n">
+        <v>148.4725</v>
+      </c>
+      <c r="G40" s="7" t="n">
+        <v>150.29</v>
+      </c>
+      <c r="H40" s="7" t="n">
+        <v>185.4425</v>
+      </c>
+      <c r="I40" s="7" t="n">
+        <v>220.2431</v>
+      </c>
+      <c r="J40" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K40" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="L40" s="6" t="inlineStr">
+        <is>
+          <t>benchmark_local_20users_run3_1790885902011.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="19" customHeight="1">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="C41" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" s="7" t="n">
+        <v>300</v>
+      </c>
+      <c r="E41" s="7" t="n">
+        <v>139.8601398601399</v>
+      </c>
+      <c r="F41" s="7" t="n">
+        <v>330.5770666666667</v>
+      </c>
+      <c r="G41" s="7" t="n">
+        <v>316.185</v>
+      </c>
+      <c r="H41" s="7" t="n">
+        <v>473.993</v>
+      </c>
+      <c r="I41" s="7" t="n">
+        <v>493.8226</v>
+      </c>
+      <c r="J41" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K41" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="L41" s="6" t="inlineStr">
+        <is>
+          <t>benchmark_local_50users_run1_1789163292223.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="19" customHeight="1">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B42" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="C42" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" s="7" t="n">
+        <v>300</v>
+      </c>
+      <c r="E42" s="7" t="n">
+        <v>1376.146788990826</v>
+      </c>
+      <c r="F42" s="7" t="n">
+        <v>39.41496666666666</v>
+      </c>
+      <c r="G42" s="7" t="n">
+        <v>38.86</v>
+      </c>
+      <c r="H42" s="7" t="n">
+        <v>57.15600000000005</v>
+      </c>
+      <c r="I42" s="7" t="n">
+        <v>71.8034</v>
+      </c>
+      <c r="J42" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="K42" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L42" s="6" t="inlineStr">
+        <is>
+          <t>benchmark_local_50users_run1_1790816141073.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="19" customHeight="1">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="C43" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" s="7" t="n">
+        <v>300</v>
+      </c>
+      <c r="E43" s="7" t="n">
+        <v>5.560601286352431</v>
+      </c>
+      <c r="F43" s="7" t="n">
+        <v>3245.659466666667</v>
+      </c>
+      <c r="G43" s="7" t="n">
+        <v>4012.765</v>
+      </c>
+      <c r="H43" s="7" t="n">
+        <v>6116.05</v>
+      </c>
+      <c r="I43" s="7" t="n">
+        <v>6117.263</v>
+      </c>
+      <c r="J43" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K43" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="L43" s="6" t="inlineStr">
+        <is>
+          <t>benchmark_local_50users_run1_1790885961760.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="19" customHeight="1">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="C44" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D44" s="7" t="n">
+        <v>300</v>
+      </c>
+      <c r="E44" s="7" t="n">
+        <v>82.23684210526315</v>
+      </c>
+      <c r="F44" s="7" t="n">
+        <v>548.6262666666667</v>
+      </c>
+      <c r="G44" s="7" t="n">
+        <v>549.4300000000001</v>
+      </c>
+      <c r="H44" s="7" t="n">
+        <v>848.922</v>
+      </c>
+      <c r="I44" s="7" t="n">
+        <v>880.3430999999999</v>
+      </c>
+      <c r="J44" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K44" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="L44" s="6" t="inlineStr">
+        <is>
+          <t>benchmark_local_50users_run2_1789163299025.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="19" customHeight="1">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="C45" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D45" s="7" t="n">
+        <v>300</v>
+      </c>
+      <c r="E45" s="7" t="n">
+        <v>1357.466063348416</v>
+      </c>
+      <c r="F45" s="7" t="n">
+        <v>39.43283333333333</v>
+      </c>
+      <c r="G45" s="7" t="n">
+        <v>37.48</v>
+      </c>
+      <c r="H45" s="7" t="n">
+        <v>64.501</v>
+      </c>
+      <c r="I45" s="7" t="n">
+        <v>78.5031</v>
+      </c>
+      <c r="J45" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="K45" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L45" s="6" t="inlineStr">
+        <is>
+          <t>benchmark_local_50users_run2_1790816146617.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="19" customHeight="1">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B46" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="C46" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D46" s="7" t="n">
+        <v>300</v>
+      </c>
+      <c r="E46" s="7" t="n">
+        <v>8.94534394847482</v>
+      </c>
+      <c r="F46" s="7" t="n">
+        <v>2210.781933333334</v>
+      </c>
+      <c r="G46" s="7" t="n">
+        <v>392.505</v>
+      </c>
+      <c r="H46" s="7" t="n">
+        <v>6110.314</v>
+      </c>
+      <c r="I46" s="7" t="n">
+        <v>6112.5704</v>
+      </c>
+      <c r="J46" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K46" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="L46" s="6" t="inlineStr">
+        <is>
+          <t>benchmark_local_50users_run2_1790886001045.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="19" customHeight="1">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="C47" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D47" s="7" t="n">
+        <v>300</v>
+      </c>
+      <c r="E47" s="7" t="n">
         <v>93.31259720062209</v>
       </c>
-      <c r="F22" s="7" t="n">
+      <c r="F47" s="7" t="n">
         <v>489.9441</v>
       </c>
-      <c r="G22" s="7" t="n">
+      <c r="G47" s="7" t="n">
         <v>528.285</v>
       </c>
-      <c r="H22" s="7" t="n">
+      <c r="H47" s="7" t="n">
         <v>656.9325</v>
       </c>
-      <c r="I22" s="7" t="n">
+      <c r="I47" s="7" t="n">
         <v>677.7666</v>
       </c>
-      <c r="J22" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K22" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="L22" s="6" t="inlineStr">
+      <c r="J47" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K47" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="L47" s="6" t="inlineStr">
         <is>
           <t>benchmark_local_50users_run3_1789163305329.csv</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+    <row r="48" ht="19" customHeight="1">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B48" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="C48" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D48" s="7" t="n">
+        <v>300</v>
+      </c>
+      <c r="E48" s="7" t="n">
+        <v>1562.5</v>
+      </c>
+      <c r="F48" s="7" t="n">
+        <v>36.31436666666667</v>
+      </c>
+      <c r="G48" s="7" t="n">
+        <v>33.495</v>
+      </c>
+      <c r="H48" s="7" t="n">
+        <v>70.66050000000001</v>
+      </c>
+      <c r="I48" s="7" t="n">
+        <v>80.05629999999999</v>
+      </c>
+      <c r="J48" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="K48" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L48" s="6" t="inlineStr">
+        <is>
+          <t>benchmark_local_50users_run3_1790816152180.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="19" customHeight="1">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="C49" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D49" s="7" t="n">
+        <v>300</v>
+      </c>
+      <c r="E49" s="7" t="n">
+        <v>6.5705900389855</v>
+      </c>
+      <c r="F49" s="7" t="n">
+        <v>2630.502466666667</v>
+      </c>
+      <c r="G49" s="7" t="n">
+        <v>2549.54</v>
+      </c>
+      <c r="H49" s="7" t="n">
+        <v>6076.929</v>
+      </c>
+      <c r="I49" s="7" t="n">
+        <v>6079.4607</v>
+      </c>
+      <c r="J49" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K49" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="L49" s="6" t="inlineStr">
+        <is>
+          <t>benchmark_local_50users_run3_1790886051556.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>Fonte: Elaborado pelos autores (2026).</t>
         </is>
@@ -2236,7 +3370,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="54" customWidth="1" min="1" max="1"/>
@@ -2364,7 +3498,7 @@
         <v>10</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D6" s="7" t="n">
         <v>20</v>
@@ -2373,20 +3507,20 @@
         <v>20.03</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>6.3</v>
+        <v>11.42</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>804.2</v>
+        <v>429.2</v>
       </c>
       <c r="H6" s="7" t="n">
-        <v>3029.2</v>
+        <v>1744.7</v>
       </c>
       <c r="I6" s="7" t="n">
         <v>100</v>
       </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
-          <t>heavy_uploads_aws_10users_run2_1789182153872.csv</t>
+          <t>heavy_uploads_aws_10users_run1_1790891065968.csv</t>
         </is>
       </c>
     </row>
@@ -2400,7 +3534,7 @@
         <v>10</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D7" s="7" t="n">
         <v>20</v>
@@ -2409,20 +3543,20 @@
         <v>20.03</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>6.69</v>
+        <v>6.3</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>365</v>
+        <v>804.2</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>1679.1</v>
+        <v>3029.2</v>
       </c>
       <c r="I7" s="7" t="n">
         <v>100</v>
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>heavy_uploads_aws_10users_run3_1789182158657.csv</t>
+          <t>heavy_uploads_aws_10users_run2_1789182153872.csv</t>
         </is>
       </c>
     </row>
@@ -2433,32 +3567,32 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="C8" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D8" s="7" t="n">
-        <v>40</v>
-      </c>
       <c r="E8" s="7" t="n">
-        <v>40.05</v>
+        <v>20.03</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>13.41</v>
+        <v>17.65</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>578.3</v>
+        <v>453.6</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>2674.9</v>
+        <v>959.4</v>
       </c>
       <c r="I8" s="7" t="n">
         <v>100</v>
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>heavy_uploads_aws_20users_run1_1789182163406.csv</t>
+          <t>heavy_uploads_aws_10users_run2_1790891068838.csv</t>
         </is>
       </c>
     </row>
@@ -2469,32 +3603,32 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D9" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="C9" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D9" s="7" t="n">
-        <v>40</v>
-      </c>
       <c r="E9" s="7" t="n">
-        <v>40.05</v>
+        <v>20.03</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>9.83</v>
+        <v>6.69</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>486.5</v>
+        <v>365</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>2332.6</v>
+        <v>1679.1</v>
       </c>
       <c r="I9" s="7" t="n">
         <v>100</v>
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>heavy_uploads_aws_20users_run2_1789182169261.csv</t>
+          <t>heavy_uploads_aws_10users_run3_1789182158657.csv</t>
         </is>
       </c>
     </row>
@@ -2505,32 +3639,32 @@
         </is>
       </c>
       <c r="B10" s="7" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C10" s="7" t="n">
         <v>3</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>40.05</v>
+        <v>20.03</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>5.05</v>
+        <v>18.08</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>596.8</v>
+        <v>374.5</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>5660.7</v>
+        <v>1088.4</v>
       </c>
       <c r="I10" s="7" t="n">
         <v>100</v>
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>heavy_uploads_aws_20users_run3_1789182178983.csv</t>
+          <t>heavy_uploads_aws_10users_run3_1790891071793.csv</t>
         </is>
       </c>
     </row>
@@ -2541,32 +3675,32 @@
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="C11" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D11" s="7" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>10.01</v>
+        <v>40.05</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>7.36</v>
+        <v>13.41</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>782.9</v>
+        <v>578.3</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>1358</v>
+        <v>2674.9</v>
       </c>
       <c r="I11" s="7" t="n">
         <v>100</v>
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>heavy_uploads_aws_5users_run1_1789182135082.csv</t>
+          <t>heavy_uploads_aws_20users_run1_1789182163406.csv</t>
         </is>
       </c>
     </row>
@@ -2577,32 +3711,32 @@
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="C12" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D12" s="7" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>10.01</v>
+        <v>40.05</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>15.56</v>
+        <v>12.22</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>369.9</v>
+        <v>523.7</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>625</v>
+        <v>2264.9</v>
       </c>
       <c r="I12" s="7" t="n">
         <v>100</v>
       </c>
       <c r="J12" s="6" t="inlineStr">
         <is>
-          <t>heavy_uploads_aws_5users_run2_1789182137494.csv</t>
+          <t>heavy_uploads_aws_20users_run1_1790891077030.csv</t>
         </is>
       </c>
     </row>
@@ -2613,262 +3747,262 @@
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="C13" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D13" s="7" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>10.01</v>
+        <v>40.05</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>18.19</v>
+        <v>9.83</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>306.1</v>
+        <v>486.5</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>516</v>
+        <v>2332.6</v>
       </c>
       <c r="I13" s="7" t="n">
         <v>100</v>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
-          <t>heavy_uploads_aws_5users_run3_1789182139763.csv</t>
+          <t>heavy_uploads_aws_20users_run2_1789182169261.csv</t>
         </is>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Local (Docker)</t>
+          <t>Nuvem (AWS)</t>
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C14" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D14" s="7" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="E14" s="7" t="n">
-        <v>20.03</v>
+        <v>40.05</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>100.85</v>
+        <v>13.64</v>
       </c>
       <c r="G14" s="7" t="n">
-        <v>126.7</v>
+        <v>461.5</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>197.5</v>
+        <v>2743.8</v>
       </c>
       <c r="I14" s="7" t="n">
         <v>100</v>
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
-          <t>heavy_uploads_local_10users_run1_1789163341337.csv</t>
+          <t>heavy_uploads_aws_20users_run2_1790891081991.csv</t>
         </is>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Local (Docker)</t>
+          <t>Nuvem (AWS)</t>
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C15" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D15" s="7" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>20.03</v>
+        <v>40.05</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>83.23</v>
+        <v>5.05</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>135.5</v>
+        <v>596.8</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>189</v>
+        <v>5660.7</v>
       </c>
       <c r="I15" s="7" t="n">
         <v>100</v>
       </c>
       <c r="J15" s="6" t="inlineStr">
         <is>
-          <t>heavy_uploads_local_10users_run2_1789163343196.csv</t>
+          <t>heavy_uploads_aws_20users_run3_1789182178983.csv</t>
         </is>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Local (Docker)</t>
+          <t>Nuvem (AWS)</t>
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C16" s="7" t="n">
         <v>3</v>
       </c>
       <c r="D16" s="7" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="E16" s="7" t="n">
-        <v>20.03</v>
+        <v>40.05</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>109.31</v>
+        <v>13.08</v>
       </c>
       <c r="G16" s="7" t="n">
-        <v>111.2</v>
+        <v>500.7</v>
       </c>
       <c r="H16" s="7" t="n">
-        <v>165.7</v>
+        <v>2789</v>
       </c>
       <c r="I16" s="7" t="n">
         <v>100</v>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
-          <t>heavy_uploads_local_10users_run3_1789163345005.csv</t>
+          <t>heavy_uploads_aws_20users_run3_1790891086987.csv</t>
         </is>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Local (Docker)</t>
+          <t>Nuvem (AWS)</t>
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="C17" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D17" s="7" t="n">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>40.05</v>
+        <v>10.01</v>
       </c>
       <c r="F17" s="7" t="n">
-        <v>80.08</v>
+        <v>7.36</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>249.9</v>
+        <v>782.9</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>341.1</v>
+        <v>1358</v>
       </c>
       <c r="I17" s="7" t="n">
         <v>100</v>
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
-          <t>heavy_uploads_local_20users_run1_1789163347250.csv</t>
+          <t>heavy_uploads_aws_5users_run1_1789182135082.csv</t>
         </is>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Local (Docker)</t>
+          <t>Nuvem (AWS)</t>
         </is>
       </c>
       <c r="B18" s="7" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="C18" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D18" s="7" t="n">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="E18" s="7" t="n">
-        <v>40.05</v>
+        <v>10.01</v>
       </c>
       <c r="F18" s="7" t="n">
-        <v>67.78</v>
+        <v>6.97</v>
       </c>
       <c r="G18" s="7" t="n">
-        <v>331.6</v>
+        <v>765.6</v>
       </c>
       <c r="H18" s="7" t="n">
-        <v>443.9</v>
+        <v>1423.6</v>
       </c>
       <c r="I18" s="7" t="n">
         <v>100</v>
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
-          <t>heavy_uploads_local_20users_run2_1789163349685.csv</t>
+          <t>heavy_uploads_aws_5users_run1_1790891057554.csv</t>
         </is>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Local (Docker)</t>
+          <t>Nuvem (AWS)</t>
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="C19" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D19" s="7" t="n">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>40.05</v>
+        <v>10.01</v>
       </c>
       <c r="F19" s="7" t="n">
-        <v>71.86</v>
+        <v>15.56</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>314.9</v>
+        <v>369.9</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>382.6</v>
+        <v>625</v>
       </c>
       <c r="I19" s="7" t="n">
         <v>100</v>
       </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
-          <t>heavy_uploads_local_20users_run3_1789163352099.csv</t>
+          <t>heavy_uploads_aws_5users_run2_1789182137494.csv</t>
         </is>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Local (Docker)</t>
+          <t>Nuvem (AWS)</t>
         </is>
       </c>
       <c r="B20" s="7" t="n">
         <v>5</v>
       </c>
       <c r="C20" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D20" s="7" t="n">
         <v>10</v>
@@ -2877,34 +4011,34 @@
         <v>10.01</v>
       </c>
       <c r="F20" s="7" t="n">
-        <v>63.46</v>
+        <v>15.91</v>
       </c>
       <c r="G20" s="7" t="n">
-        <v>81</v>
+        <v>348.2</v>
       </c>
       <c r="H20" s="7" t="n">
-        <v>144.9</v>
+        <v>618</v>
       </c>
       <c r="I20" s="7" t="n">
         <v>100</v>
       </c>
       <c r="J20" s="6" t="inlineStr">
         <is>
-          <t>heavy_uploads_local_5users_run1_1789163336068.csv</t>
+          <t>heavy_uploads_aws_5users_run2_1790891059967.csv</t>
         </is>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Local (Docker)</t>
+          <t>Nuvem (AWS)</t>
         </is>
       </c>
       <c r="B21" s="7" t="n">
         <v>5</v>
       </c>
       <c r="C21" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D21" s="7" t="n">
         <v>10</v>
@@ -2913,27 +4047,27 @@
         <v>10.01</v>
       </c>
       <c r="F21" s="7" t="n">
-        <v>72.36</v>
+        <v>18.19</v>
       </c>
       <c r="G21" s="7" t="n">
-        <v>75.5</v>
+        <v>306.1</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>129.9</v>
+        <v>516</v>
       </c>
       <c r="I21" s="7" t="n">
         <v>100</v>
       </c>
       <c r="J21" s="6" t="inlineStr">
         <is>
-          <t>heavy_uploads_local_5users_run2_1789163337774.csv</t>
+          <t>heavy_uploads_aws_5users_run3_1789182139763.csv</t>
         </is>
       </c>
     </row>
     <row r="22" ht="19" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>Local (Docker)</t>
+          <t>Nuvem (AWS)</t>
         </is>
       </c>
       <c r="B22" s="7" t="n">
@@ -2949,25 +4083,1105 @@
         <v>10.01</v>
       </c>
       <c r="F22" s="7" t="n">
+        <v>15.03</v>
+      </c>
+      <c r="G22" s="7" t="n">
+        <v>318.7</v>
+      </c>
+      <c r="H22" s="7" t="n">
+        <v>613.2</v>
+      </c>
+      <c r="I22" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J22" s="6" t="inlineStr">
+        <is>
+          <t>heavy_uploads_aws_5users_run3_1790891062353.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="19" customHeight="1">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="C23" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="E23" s="7" t="n">
+        <v>20.03</v>
+      </c>
+      <c r="F23" s="7" t="n">
+        <v>100.85</v>
+      </c>
+      <c r="G23" s="7" t="n">
+        <v>126.7</v>
+      </c>
+      <c r="H23" s="7" t="n">
+        <v>197.5</v>
+      </c>
+      <c r="I23" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J23" s="6" t="inlineStr">
+        <is>
+          <t>heavy_uploads_local_10users_run1_1789163341337.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="19" customHeight="1">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="C24" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="E24" s="7" t="n">
+        <v>20.03</v>
+      </c>
+      <c r="F24" s="7" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="G24" s="7" t="n">
+        <v>39</v>
+      </c>
+      <c r="H24" s="7" t="n">
+        <v>64594.6</v>
+      </c>
+      <c r="I24" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" s="6" t="inlineStr">
+        <is>
+          <t>heavy_uploads_local_10users_run1_1790818625316.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="19" customHeight="1">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="C25" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="E25" s="7" t="n">
+        <v>20.03</v>
+      </c>
+      <c r="F25" s="7" t="n">
+        <v>59.21</v>
+      </c>
+      <c r="G25" s="7" t="n">
+        <v>210.8</v>
+      </c>
+      <c r="H25" s="7" t="n">
+        <v>324.7</v>
+      </c>
+      <c r="I25" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J25" s="6" t="inlineStr">
+        <is>
+          <t>heavy_uploads_local_10users_run1_1790823952849.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="19" customHeight="1">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="C26" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="E26" s="7" t="n">
+        <v>20.03</v>
+      </c>
+      <c r="F26" s="7" t="n">
+        <v>44.69</v>
+      </c>
+      <c r="G26" s="7" t="n">
+        <v>152.6</v>
+      </c>
+      <c r="H26" s="7" t="n">
+        <v>383.2</v>
+      </c>
+      <c r="I26" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J26" s="6" t="inlineStr">
+        <is>
+          <t>heavy_uploads_local_10users_run1_1790886283182.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="19" customHeight="1">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="C27" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D27" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="E27" s="7" t="n">
+        <v>20.03</v>
+      </c>
+      <c r="F27" s="7" t="n">
+        <v>83.23</v>
+      </c>
+      <c r="G27" s="7" t="n">
+        <v>135.5</v>
+      </c>
+      <c r="H27" s="7" t="n">
+        <v>189</v>
+      </c>
+      <c r="I27" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J27" s="6" t="inlineStr">
+        <is>
+          <t>heavy_uploads_local_10users_run2_1789163343196.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="19" customHeight="1">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="C28" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D28" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="E28" s="7" t="n">
+        <v>20.03</v>
+      </c>
+      <c r="F28" s="7" t="n">
+        <v>159.42</v>
+      </c>
+      <c r="G28" s="7" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="H28" s="7" t="n">
+        <v>109.2</v>
+      </c>
+      <c r="I28" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" s="6" t="inlineStr">
+        <is>
+          <t>heavy_uploads_local_10users_run2_1790818628909.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="19" customHeight="1">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="C29" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D29" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="E29" s="7" t="n">
+        <v>20.03</v>
+      </c>
+      <c r="F29" s="7" t="n">
+        <v>46.37</v>
+      </c>
+      <c r="G29" s="7" t="n">
+        <v>183.4</v>
+      </c>
+      <c r="H29" s="7" t="n">
+        <v>421.5</v>
+      </c>
+      <c r="I29" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J29" s="6" t="inlineStr">
+        <is>
+          <t>heavy_uploads_local_10users_run2_1790886287304.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="19" customHeight="1">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="C30" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D30" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="E30" s="7" t="n">
+        <v>20.03</v>
+      </c>
+      <c r="F30" s="7" t="n">
+        <v>109.31</v>
+      </c>
+      <c r="G30" s="7" t="n">
+        <v>111.2</v>
+      </c>
+      <c r="H30" s="7" t="n">
+        <v>165.7</v>
+      </c>
+      <c r="I30" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J30" s="6" t="inlineStr">
+        <is>
+          <t>heavy_uploads_local_10users_run3_1789163345005.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="19" customHeight="1">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="C31" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D31" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="E31" s="7" t="n">
+        <v>20.03</v>
+      </c>
+      <c r="F31" s="7" t="n">
+        <v>128.49</v>
+      </c>
+      <c r="G31" s="7" t="n">
+        <v>28.2</v>
+      </c>
+      <c r="H31" s="7" t="n">
+        <v>124.3</v>
+      </c>
+      <c r="I31" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" s="6" t="inlineStr">
+        <is>
+          <t>heavy_uploads_local_10users_run3_1790818633289.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="19" customHeight="1">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="C32" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D32" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="E32" s="7" t="n">
+        <v>20.03</v>
+      </c>
+      <c r="F32" s="7" t="n">
+        <v>65.66</v>
+      </c>
+      <c r="G32" s="7" t="n">
+        <v>123.2</v>
+      </c>
+      <c r="H32" s="7" t="n">
+        <v>274.6</v>
+      </c>
+      <c r="I32" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J32" s="6" t="inlineStr">
+        <is>
+          <t>heavy_uploads_local_10users_run3_1790886291785.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="19" customHeight="1">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="C33" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="E33" s="7" t="n">
+        <v>40.05</v>
+      </c>
+      <c r="F33" s="7" t="n">
+        <v>80.08</v>
+      </c>
+      <c r="G33" s="7" t="n">
+        <v>249.9</v>
+      </c>
+      <c r="H33" s="7" t="n">
+        <v>341.1</v>
+      </c>
+      <c r="I33" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J33" s="6" t="inlineStr">
+        <is>
+          <t>heavy_uploads_local_20users_run1_1789163347250.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="19" customHeight="1">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="C34" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="E34" s="7" t="n">
+        <v>40.05</v>
+      </c>
+      <c r="F34" s="7" t="n">
+        <v>160.4</v>
+      </c>
+      <c r="G34" s="7" t="n">
+        <v>51.1</v>
+      </c>
+      <c r="H34" s="7" t="n">
+        <v>209.9</v>
+      </c>
+      <c r="I34" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" s="6" t="inlineStr">
+        <is>
+          <t>heavy_uploads_local_20users_run1_1790818637623.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="19" customHeight="1">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="C35" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="E35" s="7" t="n">
+        <v>40.05</v>
+      </c>
+      <c r="F35" s="7" t="n">
+        <v>15.76</v>
+      </c>
+      <c r="G35" s="7" t="n">
+        <v>383.1</v>
+      </c>
+      <c r="H35" s="7" t="n">
+        <v>558.2</v>
+      </c>
+      <c r="I35" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J35" s="6" t="inlineStr">
+        <is>
+          <t>heavy_uploads_local_20users_run1_1790824030206.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="19" customHeight="1">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="C36" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="E36" s="7" t="n">
+        <v>40.05</v>
+      </c>
+      <c r="F36" s="7" t="n">
+        <v>90.89</v>
+      </c>
+      <c r="G36" s="7" t="n">
+        <v>305.1</v>
+      </c>
+      <c r="H36" s="7" t="n">
+        <v>434.1</v>
+      </c>
+      <c r="I36" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J36" s="6" t="inlineStr">
+        <is>
+          <t>heavy_uploads_local_20users_run1_1790886295830.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="19" customHeight="1">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="C37" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D37" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="E37" s="7" t="n">
+        <v>40.05</v>
+      </c>
+      <c r="F37" s="7" t="n">
+        <v>67.78</v>
+      </c>
+      <c r="G37" s="7" t="n">
+        <v>331.6</v>
+      </c>
+      <c r="H37" s="7" t="n">
+        <v>443.9</v>
+      </c>
+      <c r="I37" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J37" s="6" t="inlineStr">
+        <is>
+          <t>heavy_uploads_local_20users_run2_1789163349685.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="19" customHeight="1">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="C38" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D38" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="E38" s="7" t="n">
+        <v>40.05</v>
+      </c>
+      <c r="F38" s="7" t="n">
+        <v>146.69</v>
+      </c>
+      <c r="G38" s="7" t="n">
+        <v>58.1</v>
+      </c>
+      <c r="H38" s="7" t="n">
+        <v>235.4</v>
+      </c>
+      <c r="I38" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J38" s="6" t="inlineStr">
+        <is>
+          <t>heavy_uploads_local_20users_run2_1790818642109.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="19" customHeight="1">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="C39" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D39" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="E39" s="7" t="n">
+        <v>40.05</v>
+      </c>
+      <c r="F39" s="7" t="n">
+        <v>54.67</v>
+      </c>
+      <c r="G39" s="7" t="n">
+        <v>259.3</v>
+      </c>
+      <c r="H39" s="7" t="n">
+        <v>688.4</v>
+      </c>
+      <c r="I39" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J39" s="6" t="inlineStr">
+        <is>
+          <t>heavy_uploads_local_20users_run2_1790886300869.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="19" customHeight="1">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="C40" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D40" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="E40" s="7" t="n">
+        <v>40.05</v>
+      </c>
+      <c r="F40" s="7" t="n">
+        <v>71.86</v>
+      </c>
+      <c r="G40" s="7" t="n">
+        <v>314.9</v>
+      </c>
+      <c r="H40" s="7" t="n">
+        <v>382.6</v>
+      </c>
+      <c r="I40" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J40" s="6" t="inlineStr">
+        <is>
+          <t>heavy_uploads_local_20users_run3_1789163352099.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="19" customHeight="1">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="C41" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D41" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="E41" s="7" t="n">
+        <v>40.05</v>
+      </c>
+      <c r="F41" s="7" t="n">
+        <v>151.16</v>
+      </c>
+      <c r="G41" s="7" t="n">
+        <v>60.7</v>
+      </c>
+      <c r="H41" s="7" t="n">
+        <v>233.6</v>
+      </c>
+      <c r="I41" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J41" s="6" t="inlineStr">
+        <is>
+          <t>heavy_uploads_local_20users_run3_1790818646554.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="19" customHeight="1">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B42" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="C42" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D42" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="E42" s="7" t="n">
+        <v>40.05</v>
+      </c>
+      <c r="F42" s="7" t="n">
+        <v>92.16</v>
+      </c>
+      <c r="G42" s="7" t="n">
+        <v>287</v>
+      </c>
+      <c r="H42" s="7" t="n">
+        <v>422.1</v>
+      </c>
+      <c r="I42" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J42" s="6" t="inlineStr">
+        <is>
+          <t>heavy_uploads_local_20users_run3_1790886305738.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="19" customHeight="1">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C43" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="E43" s="7" t="n">
+        <v>10.01</v>
+      </c>
+      <c r="F43" s="7" t="n">
+        <v>63.46</v>
+      </c>
+      <c r="G43" s="7" t="n">
+        <v>81</v>
+      </c>
+      <c r="H43" s="7" t="n">
+        <v>144.9</v>
+      </c>
+      <c r="I43" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J43" s="6" t="inlineStr">
+        <is>
+          <t>heavy_uploads_local_5users_run1_1789163336068.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="19" customHeight="1">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C44" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="E44" s="7" t="n">
+        <v>10.01</v>
+      </c>
+      <c r="F44" s="7" t="n">
+        <v>112.68</v>
+      </c>
+      <c r="G44" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="H44" s="7" t="n">
+        <v>87.3</v>
+      </c>
+      <c r="I44" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J44" s="6" t="inlineStr">
+        <is>
+          <t>heavy_uploads_local_5users_run1_1790816172806.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="19" customHeight="1">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C45" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="E45" s="7" t="n">
+        <v>10.01</v>
+      </c>
+      <c r="F45" s="7" t="n">
+        <v>36.52</v>
+      </c>
+      <c r="G45" s="7" t="n">
+        <v>134.9</v>
+      </c>
+      <c r="H45" s="7" t="n">
+        <v>270.2</v>
+      </c>
+      <c r="I45" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J45" s="6" t="inlineStr">
+        <is>
+          <t>heavy_uploads_local_5users_run1_1790823941828.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="19" customHeight="1">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B46" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C46" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="E46" s="7" t="n">
+        <v>10.01</v>
+      </c>
+      <c r="F46" s="7" t="n">
+        <v>39.29</v>
+      </c>
+      <c r="G46" s="7" t="n">
+        <v>122.7</v>
+      </c>
+      <c r="H46" s="7" t="n">
+        <v>252</v>
+      </c>
+      <c r="I46" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J46" s="6" t="inlineStr">
+        <is>
+          <t>heavy_uploads_local_5users_run1_1790886270064.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="19" customHeight="1">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C47" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D47" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="E47" s="7" t="n">
+        <v>10.01</v>
+      </c>
+      <c r="F47" s="7" t="n">
+        <v>72.36</v>
+      </c>
+      <c r="G47" s="7" t="n">
+        <v>75.5</v>
+      </c>
+      <c r="H47" s="7" t="n">
+        <v>129.9</v>
+      </c>
+      <c r="I47" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J47" s="6" t="inlineStr">
+        <is>
+          <t>heavy_uploads_local_5users_run2_1789163337774.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="19" customHeight="1">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B48" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C48" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D48" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="E48" s="7" t="n">
+        <v>10.01</v>
+      </c>
+      <c r="F48" s="7" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="G48" s="7" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="H48" s="7" t="n">
+        <v>670926.1</v>
+      </c>
+      <c r="I48" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J48" s="6" t="inlineStr">
+        <is>
+          <t>heavy_uploads_local_5users_run2_1790817397538.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="19" customHeight="1">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C49" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D49" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="E49" s="7" t="n">
+        <v>10.01</v>
+      </c>
+      <c r="F49" s="7" t="n">
+        <v>42.68</v>
+      </c>
+      <c r="G49" s="7" t="n">
+        <v>107.3</v>
+      </c>
+      <c r="H49" s="7" t="n">
+        <v>209.6</v>
+      </c>
+      <c r="I49" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J49" s="6" t="inlineStr">
+        <is>
+          <t>heavy_uploads_local_5users_run2_1790886274376.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="19" customHeight="1">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B50" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C50" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D50" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="E50" s="7" t="n">
+        <v>10.01</v>
+      </c>
+      <c r="F50" s="7" t="n">
         <v>71.88</v>
       </c>
-      <c r="G22" s="7" t="n">
+      <c r="G50" s="7" t="n">
         <v>55.1</v>
       </c>
-      <c r="H22" s="7" t="n">
+      <c r="H50" s="7" t="n">
         <v>124.2</v>
       </c>
-      <c r="I22" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="J22" s="6" t="inlineStr">
+      <c r="I50" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J50" s="6" t="inlineStr">
         <is>
           <t>heavy_uploads_local_5users_run3_1789163339486.csv</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+    <row r="51" ht="19" customHeight="1">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B51" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C51" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D51" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="E51" s="7" t="n">
+        <v>10.01</v>
+      </c>
+      <c r="F51" s="7" t="n">
+        <v>119.87</v>
+      </c>
+      <c r="G51" s="7" t="n">
+        <v>17.4</v>
+      </c>
+      <c r="H51" s="7" t="n">
+        <v>74.09999999999999</v>
+      </c>
+      <c r="I51" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J51" s="6" t="inlineStr">
+        <is>
+          <t>heavy_uploads_local_5users_run3_1790817401825.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="19" customHeight="1">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B52" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C52" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D52" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="E52" s="7" t="n">
+        <v>10.01</v>
+      </c>
+      <c r="F52" s="7" t="n">
+        <v>53.67</v>
+      </c>
+      <c r="G52" s="7" t="n">
+        <v>97.90000000000001</v>
+      </c>
+      <c r="H52" s="7" t="n">
+        <v>185.5</v>
+      </c>
+      <c r="I52" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J52" s="6" t="inlineStr">
+        <is>
+          <t>heavy_uploads_local_5users_run3_1790886278640.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
         <is>
           <t>Fonte: Elaborado pelos autores (2026).</t>
         </is>
@@ -2984,7 +5198,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="43" customWidth="1" min="1" max="1"/>
@@ -3117,77 +5331,293 @@
     <row r="8" ht="19" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Local (Docker)</t>
+          <t>Nuvem (AWS)</t>
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>1475.3</v>
+        <v>2379.3</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>70.2</v>
+        <v>282</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>677.9</v>
+        <v>528.9</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>75.7</v>
+        <v>0</v>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>2026-09-11T21:49:17.437Z</t>
+          <t>2026-10-01T21:44:59.137Z</t>
         </is>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Local (Docker)</t>
+          <t>Nuvem (AWS)</t>
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>1817.1</v>
+        <v>1879.3</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>66.5</v>
+        <v>233.6</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>662.1</v>
+        <v>308.8</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>45.5</v>
+        <v>0</v>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>2026-09-11T21:49:22.820Z</t>
+          <t>2026-10-01T21:45:04.655Z</t>
         </is>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Local (Docker)</t>
+          <t>Nuvem (AWS)</t>
         </is>
       </c>
       <c r="B10" s="7" t="n">
+        <v>1665.8</v>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>214.3</v>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>318</v>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01T21:45:09.743Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="19" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="n">
+        <v>1475.3</v>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>70.2</v>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>677.9</v>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>75.7</v>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-11T21:49:17.437Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="19" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="n">
+        <v>1817.1</v>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>66.5</v>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>662.1</v>
+      </c>
+      <c r="E12" s="7" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-11T21:49:22.820Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="19" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="n">
         <v>1638.3</v>
       </c>
-      <c r="C10" s="7" t="n">
+      <c r="C13" s="7" t="n">
         <v>51.6</v>
       </c>
-      <c r="D10" s="7" t="n">
+      <c r="D13" s="7" t="n">
         <v>625.9</v>
       </c>
-      <c r="E10" s="7" t="n">
+      <c r="E13" s="7" t="n">
         <v>41.3</v>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>2026-09-11T21:49:27.540Z</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="14" ht="19" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="n">
+        <v>12707</v>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>62.9</v>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>10155.7</v>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01T03:04:02.905Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="19" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="n">
+        <v>26488</v>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>93.59999999999999</v>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>8027.8</v>
+      </c>
+      <c r="E15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01T03:11:20.725Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="19" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="n">
+        <v>26850.6</v>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>61.3</v>
+      </c>
+      <c r="D16" s="7" t="n">
+        <v>8010.3</v>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01T20:16:56.155Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="19" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="n">
+        <v>8400.9</v>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>64.7</v>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>8050.4</v>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01T20:27:58.554Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="19" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="n">
+        <v>8589.200000000001</v>
+      </c>
+      <c r="C18" s="7" t="n">
+        <v>59</v>
+      </c>
+      <c r="D18" s="7" t="n">
+        <v>8130.2</v>
+      </c>
+      <c r="E18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01T20:30:47.358Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="19" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Local (Docker)</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="n">
+        <v>9006.4</v>
+      </c>
+      <c r="C19" s="7" t="n">
+        <v>70.90000000000001</v>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>8079.7</v>
+      </c>
+      <c r="E19" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01T20:33:36.519Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Fonte: Elaborado pelos autores (2026).</t>
         </is>

</xml_diff>